<commit_message>
Consolidado de pregutas frecuentes
</commit_message>
<xml_diff>
--- a/Morosos/informe_cartas_y_juntas.xlsx
+++ b/Morosos/informe_cartas_y_juntas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="209">
   <si>
     <t>dia_cita</t>
   </si>
@@ -55,16 +55,16 @@
     <t>pensiones pendientes</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>Julio</t>
+    <t>25</t>
+  </si>
+  <si>
+    <t>julio</t>
   </si>
   <si>
     <t>Liliana María García Marín</t>
   </si>
   <si>
-    <t>7 julio de 2026</t>
+    <t>21 julio de 2026</t>
   </si>
   <si>
     <t>Biblioteca</t>
@@ -76,12 +76,30 @@
     <t>Alzate Monsalve David</t>
   </si>
   <si>
+    <t>Arango Salazar Luciana</t>
+  </si>
+  <si>
+    <t>Arango Salazar Ximena</t>
+  </si>
+  <si>
     <t>Arenas Calderon Evoleth</t>
   </si>
   <si>
     <t>Arenas Calderon Salomon</t>
   </si>
   <si>
+    <t>Artunduaga Burgos Emmanuel</t>
+  </si>
+  <si>
+    <t>Artunduaga Burgos Isaac</t>
+  </si>
+  <si>
+    <t>Artunduaga Burgos Sarahy</t>
+  </si>
+  <si>
+    <t>Cardona Mosquera Isaac</t>
+  </si>
+  <si>
     <t>Cardona Mosquera Roxana</t>
   </si>
   <si>
@@ -91,27 +109,66 @@
     <t>Cortes Correa Rebeca</t>
   </si>
   <si>
+    <t>Cortes Correa Salome</t>
+  </si>
+  <si>
+    <t>Cuervo Consuegra Tamara</t>
+  </si>
+  <si>
+    <t>Diaz Gonzalez Matias</t>
+  </si>
+  <si>
+    <t>Echeverri Agudelo Samuel</t>
+  </si>
+  <si>
     <t>Garcia Ramirez Nicolas</t>
   </si>
   <si>
     <t>Garcia Ramirez Thomás</t>
   </si>
   <si>
+    <t>Guette Ortiz Ashley Carolina</t>
+  </si>
+  <si>
+    <t>Guette Ortiz Norah Isabella</t>
+  </si>
+  <si>
+    <t>Jaramillo Agudelo Ana Sofia</t>
+  </si>
+  <si>
     <t>Luna Rincon Juan Sebastian</t>
   </si>
   <si>
     <t>Machado Taborda Mateo</t>
   </si>
   <si>
+    <t>Manco Fonnegra Samuel</t>
+  </si>
+  <si>
+    <t>Marin Vergara Nicolas</t>
+  </si>
+  <si>
     <t>Martinez Alvarez Thiago</t>
   </si>
   <si>
     <t>Martinez Ciro Josue</t>
   </si>
   <si>
+    <t>Martinez Correa Tomas</t>
+  </si>
+  <si>
     <t>Mesa Cardona Mariangel</t>
   </si>
   <si>
+    <t>Montoya Crumb Ahavah Joy</t>
+  </si>
+  <si>
+    <t>Montoya Crumb Aviva Faith</t>
+  </si>
+  <si>
+    <t>Montoya Crumb Samuel Robert</t>
+  </si>
+  <si>
     <t>Muñoz Vellojin Mateo</t>
   </si>
   <si>
@@ -121,21 +178,48 @@
     <t>Ortiz Cano Sara</t>
   </si>
   <si>
+    <t>Perez Pino Susana</t>
+  </si>
+  <si>
     <t>Pérez Hernández Salomé</t>
   </si>
   <si>
+    <t>Ramirez Avila Daniel</t>
+  </si>
+  <si>
+    <t>Ramirez Avila Sara</t>
+  </si>
+  <si>
     <t>Restrepo Cortes Isabella</t>
   </si>
   <si>
     <t>Restrepo Cortes Juan Manuel</t>
   </si>
   <si>
+    <t>Rizo Paez David Armando</t>
+  </si>
+  <si>
+    <t>Rizo Paez Elisa Victoria</t>
+  </si>
+  <si>
+    <t>Ruiz Aristizabal Nicolas</t>
+  </si>
+  <si>
+    <t>Ruiz Estrada Sofia Camila</t>
+  </si>
+  <si>
+    <t>Ruiz Rodas Jacobo</t>
+  </si>
+  <si>
     <t>Sanabria Cardona Santiago</t>
   </si>
   <si>
     <t>Sanchez Bustamante Genesis</t>
   </si>
   <si>
+    <t>Sanchez Bustamante Manuela</t>
+  </si>
+  <si>
     <t>Sanchez Bustamante Sarah Joann</t>
   </si>
   <si>
@@ -151,13 +235,19 @@
     <t>Segura Rios Samuel Felipe</t>
   </si>
   <si>
+    <t>Serna Ramirez Luciana</t>
+  </si>
+  <si>
     <t>Sierra Peñaranda Miguel Angel</t>
   </si>
   <si>
+    <t>Tenorio Maya Liam</t>
+  </si>
+  <si>
     <t>Troya Rendon Emanuel</t>
   </si>
   <si>
-    <t>Vanegas Olaya Simon</t>
+    <t>Vanegas Pulgarin Sheray</t>
   </si>
   <si>
     <t>Vasquez Rodas Josue</t>
@@ -166,15 +256,36 @@
     <t>Velez Ortiz Simon</t>
   </si>
   <si>
+    <t>Zapata Echeverry Abigail</t>
+  </si>
+  <si>
     <t>1036521142</t>
   </si>
   <si>
+    <t>1025661559</t>
+  </si>
+  <si>
+    <t>1035424821</t>
+  </si>
+  <si>
     <t>1020229348</t>
   </si>
   <si>
     <t>1011519538</t>
   </si>
   <si>
+    <t>1020322501</t>
+  </si>
+  <si>
+    <t>1020327607</t>
+  </si>
+  <si>
+    <t>1020317655</t>
+  </si>
+  <si>
+    <t>1013464926</t>
+  </si>
+  <si>
     <t>1013466654</t>
   </si>
   <si>
@@ -184,27 +295,66 @@
     <t>1025898446</t>
   </si>
   <si>
+    <t>1025895387</t>
+  </si>
+  <si>
+    <t>1035003747</t>
+  </si>
+  <si>
+    <t>1021930204</t>
+  </si>
+  <si>
+    <t>1011515086</t>
+  </si>
+  <si>
     <t>1013353521</t>
   </si>
   <si>
     <t>1013362371</t>
   </si>
   <si>
+    <t>1042587012</t>
+  </si>
+  <si>
+    <t>1018269052</t>
+  </si>
+  <si>
+    <t>1041634370</t>
+  </si>
+  <si>
     <t>1013350043</t>
   </si>
   <si>
     <t>1021931357</t>
   </si>
   <si>
+    <t>1020308169</t>
+  </si>
+  <si>
+    <t>1018271477</t>
+  </si>
+  <si>
     <t>1025899613</t>
   </si>
   <si>
     <t>1035005666</t>
   </si>
   <si>
+    <t>1020225476</t>
+  </si>
+  <si>
     <t>1025770324</t>
   </si>
   <si>
+    <t>1025776867</t>
+  </si>
+  <si>
+    <t>1013377365</t>
+  </si>
+  <si>
+    <t>1013370057</t>
+  </si>
+  <si>
     <t>1020307672</t>
   </si>
   <si>
@@ -214,21 +364,48 @@
     <t>1020239882</t>
   </si>
   <si>
+    <t>1020323103</t>
+  </si>
+  <si>
     <t>1020312315</t>
   </si>
   <si>
+    <t>1020226915</t>
+  </si>
+  <si>
+    <t>1016601695</t>
+  </si>
+  <si>
     <t>1015079466</t>
   </si>
   <si>
     <t>1015077703</t>
   </si>
   <si>
+    <t>1096705038</t>
+  </si>
+  <si>
+    <t>1018273200</t>
+  </si>
+  <si>
+    <t>1025895823</t>
+  </si>
+  <si>
+    <t>1013368945</t>
+  </si>
+  <si>
+    <t>1015075125</t>
+  </si>
+  <si>
     <t>1035008500</t>
   </si>
   <si>
     <t>1011404208</t>
   </si>
   <si>
+    <t>1022004383</t>
+  </si>
+  <si>
     <t>1011410559</t>
   </si>
   <si>
@@ -244,13 +421,19 @@
     <t>1141719278</t>
   </si>
   <si>
+    <t>1035978921</t>
+  </si>
+  <si>
     <t>1092540648</t>
   </si>
   <si>
+    <t>1084474489</t>
+  </si>
+  <si>
     <t>1025667898</t>
   </si>
   <si>
-    <t>1025901666</t>
+    <t>1034925183</t>
   </si>
   <si>
     <t>1034924450</t>
@@ -259,12 +442,21 @@
     <t>1025900606</t>
   </si>
   <si>
+    <t>1023655835</t>
+  </si>
+  <si>
     <t>Alzate Villa William</t>
   </si>
   <si>
+    <t>Castellanos Pinoz Johan Mateo</t>
+  </si>
+  <si>
     <t>Arenas Villa Harold Alexander</t>
   </si>
   <si>
+    <t>Artunduaga Cabrera Anderson</t>
+  </si>
+  <si>
     <t>Mosquera Rodriguez Tania Karina</t>
   </si>
   <si>
@@ -274,27 +466,54 @@
     <t>Cortes Velasquez Juan Pablo</t>
   </si>
   <si>
+    <t>Cuervo Paternina Eder Andres</t>
+  </si>
+  <si>
+    <t>Diaz Rico John Edwin</t>
+  </si>
+  <si>
+    <t>Echeverry Agudelo Sara Catalina</t>
+  </si>
+  <si>
     <t>Ramirez Suarez Leidy Tatiana</t>
   </si>
   <si>
     <t>Garcia Valencia Cesar Augusto</t>
   </si>
   <si>
+    <t>Ortiz Julio Sirly Dayana</t>
+  </si>
+  <si>
+    <t>Agudelo Torres Sumilde Elena</t>
+  </si>
+  <si>
     <t>Rincon Lopera Liliana Maria</t>
   </si>
   <si>
     <t>Sas Inversiones Myt</t>
   </si>
   <si>
+    <t>Manco Echavarria Reynel De Jesus</t>
+  </si>
+  <si>
+    <t>Vergara Mejia Sara Valentina</t>
+  </si>
+  <si>
     <t>Hernandez Morelo Liliana</t>
   </si>
   <si>
     <t>Martinez Moreno Devinson</t>
   </si>
   <si>
+    <t>Correa Mejia Catalina</t>
+  </si>
+  <si>
     <t>Cardona Gaviria Maribel</t>
   </si>
   <si>
+    <t>Montoya Diaz Luis Fernando</t>
+  </si>
+  <si>
     <t>Vellojin Cavadia Tania Marjolia</t>
   </si>
   <si>
@@ -304,12 +523,30 @@
     <t>Cano Guarin Sandra Milena</t>
   </si>
   <si>
+    <t>Perez Toro Juan Pablo</t>
+  </si>
+  <si>
     <t>Hernandez Cardona Mauricio</t>
   </si>
   <si>
+    <t>Ramirez Urrutia Fredy</t>
+  </si>
+  <si>
     <t>Restrepo Silva Jeison</t>
   </si>
   <si>
+    <t>Rizo Ibanez Jorge Armando</t>
+  </si>
+  <si>
+    <t>Agudelo Ruiz Sergio Mario</t>
+  </si>
+  <si>
+    <t>Estrada Colon Yerica Del Carmen</t>
+  </si>
+  <si>
+    <t>Rodas Marin Monica Janeth</t>
+  </si>
+  <si>
     <t>Sanabria Ballen Andres Leonardo</t>
   </si>
   <si>
@@ -328,13 +565,19 @@
     <t>Segura Camacho Oscar Dario</t>
   </si>
   <si>
+    <t>Arboleda Ramirez Daniel Andres</t>
+  </si>
+  <si>
     <t>Hernandez Ospina Juan Camilo</t>
   </si>
   <si>
+    <t>Marin Osorio Johny Alexander</t>
+  </si>
+  <si>
     <t>Troya Osorio Manuel Enrique</t>
   </si>
   <si>
-    <t>Olaya Rojas Liliana Maria</t>
+    <t>Vanegas Zuñiga Ray Andres</t>
   </si>
   <si>
     <t>Vasquez Gomez Alejandro</t>
@@ -343,15 +586,33 @@
     <t>Ortiz Velez Laura Catalina</t>
   </si>
   <si>
+    <t>Echeverry Giraldo Estefania</t>
+  </si>
+  <si>
     <t>CUARTO</t>
   </si>
   <si>
+    <t>DÉCIMO</t>
+  </si>
+  <si>
+    <t>ONCE</t>
+  </si>
+  <si>
     <t>OCTAVO</t>
   </si>
   <si>
     <t>SEGUNDO</t>
   </si>
   <si>
+    <t>QUINTO</t>
+  </si>
+  <si>
+    <t>TRANSICIÓN</t>
+  </si>
+  <si>
+    <t>SEPTIMO</t>
+  </si>
+  <si>
     <t>SEXTO</t>
   </si>
   <si>
@@ -361,28 +622,25 @@
     <t>NOVENO</t>
   </si>
   <si>
-    <t>SEPTIMO</t>
-  </si>
-  <si>
-    <t>DÉCIMO</t>
-  </si>
-  <si>
     <t>PRIMERO</t>
   </si>
   <si>
-    <t>QUINTO</t>
-  </si>
-  <si>
-    <t>Mayo - Junio</t>
-  </si>
-  <si>
-    <t>Abril - Mayo - Junio</t>
-  </si>
-  <si>
-    <t>Marzo - Abril - Mayo - Junio</t>
-  </si>
-  <si>
-    <t>Febrero - Marzo - Abril - Mayo - Junio</t>
+    <t>PRE-JARDIN</t>
+  </si>
+  <si>
+    <t>Junio - Julio</t>
+  </si>
+  <si>
+    <t>Abril - Mayo - Junio - Julio</t>
+  </si>
+  <si>
+    <t>Marzo - Abril - Mayo - Junio - Julio</t>
+  </si>
+  <si>
+    <t>Mayo - Junio - Julio</t>
+  </si>
+  <si>
+    <t>Febrero - Marzo - Abril - Mayo - Junio - Julio</t>
   </si>
 </sst>
 </file>
@@ -740,7 +998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
@@ -810,19 +1068,19 @@
         <v>19</v>
       </c>
       <c r="I2" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="J2" t="s">
-        <v>81</v>
+        <v>143</v>
       </c>
       <c r="K2" t="s">
-        <v>109</v>
+        <v>191</v>
       </c>
       <c r="L2">
-        <v>1157380</v>
+        <v>1157256</v>
       </c>
       <c r="M2" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -851,19 +1109,19 @@
         <v>20</v>
       </c>
       <c r="I3" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="J3" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="K3" t="s">
-        <v>110</v>
+        <v>192</v>
       </c>
       <c r="L3">
-        <v>1514160</v>
+        <v>956502</v>
       </c>
       <c r="M3" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -892,19 +1150,19 @@
         <v>21</v>
       </c>
       <c r="I4" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="J4" t="s">
-        <v>82</v>
+        <v>144</v>
       </c>
       <c r="K4" t="s">
-        <v>111</v>
+        <v>193</v>
       </c>
       <c r="L4">
-        <v>1899990</v>
+        <v>913296</v>
       </c>
       <c r="M4" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -933,19 +1191,19 @@
         <v>22</v>
       </c>
       <c r="I5" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="J5" t="s">
-        <v>83</v>
+        <v>145</v>
       </c>
       <c r="K5" t="s">
-        <v>111</v>
+        <v>194</v>
       </c>
       <c r="L5">
-        <v>2138976</v>
+        <v>2022880</v>
       </c>
       <c r="M5" t="s">
-        <v>120</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -974,19 +1232,19 @@
         <v>23</v>
       </c>
       <c r="I6" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="J6" t="s">
-        <v>84</v>
+        <v>145</v>
       </c>
       <c r="K6" t="s">
-        <v>109</v>
+        <v>195</v>
       </c>
       <c r="L6">
-        <v>1084856</v>
+        <v>2537320</v>
       </c>
       <c r="M6" t="s">
-        <v>119</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1015,19 +1273,19 @@
         <v>24</v>
       </c>
       <c r="I7" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J7" t="s">
-        <v>85</v>
+        <v>146</v>
       </c>
       <c r="K7" t="s">
-        <v>110</v>
+        <v>196</v>
       </c>
       <c r="L7">
-        <v>1514160</v>
+        <v>1258720</v>
       </c>
       <c r="M7" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1056,19 +1314,19 @@
         <v>25</v>
       </c>
       <c r="I8" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="J8" t="s">
-        <v>86</v>
+        <v>146</v>
       </c>
       <c r="K8" t="s">
-        <v>112</v>
+        <v>197</v>
       </c>
       <c r="L8">
-        <v>1360262</v>
+        <v>1229346</v>
       </c>
       <c r="M8" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1097,19 +1355,19 @@
         <v>26</v>
       </c>
       <c r="I9" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="J9" t="s">
-        <v>87</v>
+        <v>146</v>
       </c>
       <c r="K9" t="s">
-        <v>113</v>
+        <v>198</v>
       </c>
       <c r="L9">
-        <v>2194495</v>
+        <v>1198148</v>
       </c>
       <c r="M9" t="s">
-        <v>121</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1138,19 +1396,19 @@
         <v>27</v>
       </c>
       <c r="I10" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="J10" t="s">
-        <v>88</v>
+        <v>147</v>
       </c>
       <c r="K10" t="s">
-        <v>114</v>
+        <v>199</v>
       </c>
       <c r="L10">
-        <v>2164120</v>
+        <v>1242434</v>
       </c>
       <c r="M10" t="s">
-        <v>121</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1179,19 +1437,19 @@
         <v>28</v>
       </c>
       <c r="I11" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="J11" t="s">
-        <v>89</v>
+        <v>147</v>
       </c>
       <c r="K11" t="s">
-        <v>114</v>
+        <v>195</v>
       </c>
       <c r="L11">
-        <v>1715680</v>
+        <v>2855968</v>
       </c>
       <c r="M11" t="s">
-        <v>120</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -1220,19 +1478,19 @@
         <v>29</v>
       </c>
       <c r="I12" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="J12" t="s">
-        <v>90</v>
+        <v>148</v>
       </c>
       <c r="K12" t="s">
-        <v>115</v>
+        <v>191</v>
       </c>
       <c r="L12">
-        <v>1198148</v>
+        <v>1080284</v>
       </c>
       <c r="M12" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1261,19 +1519,19 @@
         <v>30</v>
       </c>
       <c r="I13" t="s">
-        <v>61</v>
+        <v>92</v>
       </c>
       <c r="J13" t="s">
-        <v>91</v>
+        <v>149</v>
       </c>
       <c r="K13" t="s">
-        <v>112</v>
+        <v>194</v>
       </c>
       <c r="L13">
-        <v>1762458</v>
+        <v>2022880</v>
       </c>
       <c r="M13" t="s">
-        <v>120</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1302,19 +1560,19 @@
         <v>31</v>
       </c>
       <c r="I14" t="s">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="J14" t="s">
-        <v>92</v>
+        <v>149</v>
       </c>
       <c r="K14" t="s">
-        <v>112</v>
+        <v>193</v>
       </c>
       <c r="L14">
-        <v>1096770</v>
+        <v>913296</v>
       </c>
       <c r="M14" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -1343,19 +1601,19 @@
         <v>32</v>
       </c>
       <c r="I15" t="s">
-        <v>63</v>
+        <v>94</v>
       </c>
       <c r="J15" t="s">
-        <v>93</v>
+        <v>150</v>
       </c>
       <c r="K15" t="s">
-        <v>116</v>
+        <v>198</v>
       </c>
       <c r="L15">
-        <v>2556650</v>
+        <v>1265122</v>
       </c>
       <c r="M15" t="s">
-        <v>122</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -1384,19 +1642,19 @@
         <v>33</v>
       </c>
       <c r="I16" t="s">
-        <v>64</v>
+        <v>95</v>
       </c>
       <c r="J16" t="s">
-        <v>94</v>
+        <v>151</v>
       </c>
       <c r="K16" t="s">
-        <v>109</v>
+        <v>192</v>
       </c>
       <c r="L16">
-        <v>814324</v>
+        <v>956502</v>
       </c>
       <c r="M16" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1425,19 +1683,19 @@
         <v>34</v>
       </c>
       <c r="I17" t="s">
-        <v>65</v>
+        <v>96</v>
       </c>
       <c r="J17" t="s">
-        <v>95</v>
+        <v>152</v>
       </c>
       <c r="K17" t="s">
-        <v>117</v>
+        <v>192</v>
       </c>
       <c r="L17">
-        <v>1044902</v>
+        <v>1136976</v>
       </c>
       <c r="M17" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1466,19 +1724,19 @@
         <v>35</v>
       </c>
       <c r="I18" t="s">
-        <v>66</v>
+        <v>97</v>
       </c>
       <c r="J18" t="s">
-        <v>96</v>
+        <v>153</v>
       </c>
       <c r="K18" t="s">
-        <v>110</v>
+        <v>199</v>
       </c>
       <c r="L18">
-        <v>2428600</v>
+        <v>1917016</v>
       </c>
       <c r="M18" t="s">
-        <v>122</v>
+        <v>205</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -1507,19 +1765,19 @@
         <v>36</v>
       </c>
       <c r="I19" t="s">
-        <v>67</v>
+        <v>98</v>
       </c>
       <c r="J19" t="s">
-        <v>97</v>
+        <v>154</v>
       </c>
       <c r="K19" t="s">
-        <v>113</v>
+        <v>200</v>
       </c>
       <c r="L19">
-        <v>1233196</v>
+        <v>2807794</v>
       </c>
       <c r="M19" t="s">
-        <v>120</v>
+        <v>206</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1548,19 +1806,19 @@
         <v>37</v>
       </c>
       <c r="I20" t="s">
-        <v>68</v>
+        <v>99</v>
       </c>
       <c r="J20" t="s">
-        <v>97</v>
+        <v>155</v>
       </c>
       <c r="K20" t="s">
-        <v>110</v>
+        <v>193</v>
       </c>
       <c r="L20">
-        <v>1022880</v>
+        <v>970440</v>
       </c>
       <c r="M20" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -1589,19 +1847,19 @@
         <v>38</v>
       </c>
       <c r="I21" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="J21" t="s">
-        <v>98</v>
+        <v>155</v>
       </c>
       <c r="K21" t="s">
-        <v>109</v>
+        <v>200</v>
       </c>
       <c r="L21">
-        <v>1155620</v>
+        <v>1288964</v>
       </c>
       <c r="M21" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -1630,19 +1888,19 @@
         <v>39</v>
       </c>
       <c r="I22" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="J22" t="s">
-        <v>99</v>
+        <v>156</v>
       </c>
       <c r="K22" t="s">
-        <v>114</v>
+        <v>192</v>
       </c>
       <c r="L22">
-        <v>1014246</v>
+        <v>952506</v>
       </c>
       <c r="M22" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1671,19 +1929,19 @@
         <v>40</v>
       </c>
       <c r="I23" t="s">
-        <v>71</v>
+        <v>102</v>
       </c>
       <c r="J23" t="s">
-        <v>99</v>
+        <v>157</v>
       </c>
       <c r="K23" t="s">
-        <v>112</v>
+        <v>201</v>
       </c>
       <c r="L23">
-        <v>1103508</v>
+        <v>2710150</v>
       </c>
       <c r="M23" t="s">
-        <v>119</v>
+        <v>206</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -1712,19 +1970,19 @@
         <v>41</v>
       </c>
       <c r="I24" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="J24" t="s">
-        <v>100</v>
+        <v>158</v>
       </c>
       <c r="K24" t="s">
-        <v>113</v>
+        <v>201</v>
       </c>
       <c r="L24">
-        <v>2044495</v>
+        <v>1133616</v>
       </c>
       <c r="M24" t="s">
-        <v>121</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -1753,19 +2011,19 @@
         <v>42</v>
       </c>
       <c r="I25" t="s">
-        <v>73</v>
+        <v>104</v>
       </c>
       <c r="J25" t="s">
-        <v>101</v>
+        <v>159</v>
       </c>
       <c r="K25" t="s">
-        <v>111</v>
+        <v>192</v>
       </c>
       <c r="L25">
-        <v>3574960</v>
+        <v>955753</v>
       </c>
       <c r="M25" t="s">
-        <v>122</v>
+        <v>204</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -1794,19 +2052,19 @@
         <v>43</v>
       </c>
       <c r="I26" t="s">
-        <v>74</v>
+        <v>105</v>
       </c>
       <c r="J26" t="s">
-        <v>102</v>
+        <v>160</v>
       </c>
       <c r="K26" t="s">
-        <v>110</v>
+        <v>202</v>
       </c>
       <c r="L26">
-        <v>1704306</v>
+        <v>1044902</v>
       </c>
       <c r="M26" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -1835,19 +2093,19 @@
         <v>44</v>
       </c>
       <c r="I27" t="s">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="J27" t="s">
-        <v>103</v>
+        <v>161</v>
       </c>
       <c r="K27" t="s">
-        <v>116</v>
+        <v>198</v>
       </c>
       <c r="L27">
-        <v>1016660</v>
+        <v>1198148</v>
       </c>
       <c r="M27" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -1876,19 +2134,19 @@
         <v>45</v>
       </c>
       <c r="I28" t="s">
-        <v>76</v>
+        <v>107</v>
       </c>
       <c r="J28" t="s">
-        <v>104</v>
+        <v>162</v>
       </c>
       <c r="K28" t="s">
-        <v>110</v>
+        <v>199</v>
       </c>
       <c r="L28">
-        <v>1462880</v>
+        <v>2353944</v>
       </c>
       <c r="M28" t="s">
-        <v>120</v>
+        <v>205</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -1917,19 +2175,19 @@
         <v>46</v>
       </c>
       <c r="I29" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="J29" t="s">
-        <v>105</v>
+        <v>163</v>
       </c>
       <c r="K29" t="s">
-        <v>110</v>
+        <v>193</v>
       </c>
       <c r="L29">
-        <v>2331074</v>
+        <v>969160</v>
       </c>
       <c r="M29" t="s">
-        <v>122</v>
+        <v>204</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -1958,19 +2216,19 @@
         <v>47</v>
       </c>
       <c r="I30" t="s">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="J30" t="s">
-        <v>106</v>
+        <v>164</v>
       </c>
       <c r="K30" t="s">
-        <v>118</v>
+        <v>199</v>
       </c>
       <c r="L30">
-        <v>1996644</v>
+        <v>1651524</v>
       </c>
       <c r="M30" t="s">
-        <v>120</v>
+        <v>207</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -1999,19 +2257,19 @@
         <v>48</v>
       </c>
       <c r="I31" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
       <c r="J31" t="s">
-        <v>107</v>
+        <v>165</v>
       </c>
       <c r="K31" t="s">
-        <v>112</v>
+        <v>203</v>
       </c>
       <c r="L31">
-        <v>1172972</v>
+        <v>1416696</v>
       </c>
       <c r="M31" t="s">
-        <v>119</v>
+        <v>204</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -2040,19 +2298,1290 @@
         <v>49</v>
       </c>
       <c r="I32" t="s">
+        <v>111</v>
+      </c>
+      <c r="J32" t="s">
+        <v>165</v>
+      </c>
+      <c r="K32" t="s">
+        <v>197</v>
+      </c>
+      <c r="L32">
+        <v>1160620</v>
+      </c>
+      <c r="M32" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
+      <c r="A33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33">
+        <v>2026</v>
+      </c>
+      <c r="D33" t="s">
+        <v>15</v>
+      </c>
+      <c r="E33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F33" t="s">
+        <v>17</v>
+      </c>
+      <c r="G33" t="s">
+        <v>18</v>
+      </c>
+      <c r="H33" t="s">
+        <v>50</v>
+      </c>
+      <c r="I33" t="s">
+        <v>112</v>
+      </c>
+      <c r="J33" t="s">
+        <v>165</v>
+      </c>
+      <c r="K33" t="s">
+        <v>195</v>
+      </c>
+      <c r="L33">
+        <v>1344322</v>
+      </c>
+      <c r="M33" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
+      <c r="A34" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34">
+        <v>2026</v>
+      </c>
+      <c r="D34" t="s">
+        <v>15</v>
+      </c>
+      <c r="E34" t="s">
+        <v>16</v>
+      </c>
+      <c r="F34" t="s">
+        <v>17</v>
+      </c>
+      <c r="G34" t="s">
+        <v>18</v>
+      </c>
+      <c r="H34" t="s">
+        <v>51</v>
+      </c>
+      <c r="I34" t="s">
+        <v>113</v>
+      </c>
+      <c r="J34" t="s">
+        <v>166</v>
+      </c>
+      <c r="K34" t="s">
+        <v>192</v>
+      </c>
+      <c r="L34">
+        <v>3073980</v>
+      </c>
+      <c r="M34" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
+      <c r="A35" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35">
+        <v>2026</v>
+      </c>
+      <c r="D35" t="s">
+        <v>15</v>
+      </c>
+      <c r="E35" t="s">
+        <v>16</v>
+      </c>
+      <c r="F35" t="s">
+        <v>17</v>
+      </c>
+      <c r="G35" t="s">
+        <v>18</v>
+      </c>
+      <c r="H35" t="s">
+        <v>52</v>
+      </c>
+      <c r="I35" t="s">
+        <v>114</v>
+      </c>
+      <c r="J35" t="s">
+        <v>167</v>
+      </c>
+      <c r="K35" t="s">
+        <v>191</v>
+      </c>
+      <c r="L35">
+        <v>815648</v>
+      </c>
+      <c r="M35" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
+      <c r="A36" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36">
+        <v>2026</v>
+      </c>
+      <c r="D36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E36" t="s">
+        <v>16</v>
+      </c>
+      <c r="F36" t="s">
+        <v>17</v>
+      </c>
+      <c r="G36" t="s">
+        <v>18</v>
+      </c>
+      <c r="H36" t="s">
+        <v>53</v>
+      </c>
+      <c r="I36" t="s">
+        <v>115</v>
+      </c>
+      <c r="J36" t="s">
+        <v>168</v>
+      </c>
+      <c r="K36" t="s">
+        <v>202</v>
+      </c>
+      <c r="L36">
+        <v>1190353</v>
+      </c>
+      <c r="M36" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37">
+        <v>2026</v>
+      </c>
+      <c r="D37" t="s">
+        <v>15</v>
+      </c>
+      <c r="E37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G37" t="s">
+        <v>18</v>
+      </c>
+      <c r="H37" t="s">
+        <v>54</v>
+      </c>
+      <c r="I37" t="s">
+        <v>116</v>
+      </c>
+      <c r="J37" t="s">
+        <v>169</v>
+      </c>
+      <c r="K37" t="s">
+        <v>191</v>
+      </c>
+      <c r="L37">
+        <v>1224620</v>
+      </c>
+      <c r="M37" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
+      <c r="A38" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38">
+        <v>2026</v>
+      </c>
+      <c r="D38" t="s">
+        <v>15</v>
+      </c>
+      <c r="E38" t="s">
+        <v>16</v>
+      </c>
+      <c r="F38" t="s">
+        <v>17</v>
+      </c>
+      <c r="G38" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" t="s">
+        <v>55</v>
+      </c>
+      <c r="I38" t="s">
+        <v>117</v>
+      </c>
+      <c r="J38" t="s">
+        <v>170</v>
+      </c>
+      <c r="K38" t="s">
+        <v>194</v>
+      </c>
+      <c r="L38">
+        <v>2941320</v>
+      </c>
+      <c r="M38" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
+      <c r="A39" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39">
+        <v>2026</v>
+      </c>
+      <c r="D39" t="s">
+        <v>15</v>
+      </c>
+      <c r="E39" t="s">
+        <v>16</v>
+      </c>
+      <c r="F39" t="s">
+        <v>17</v>
+      </c>
+      <c r="G39" t="s">
+        <v>18</v>
+      </c>
+      <c r="H39" t="s">
+        <v>56</v>
+      </c>
+      <c r="I39" t="s">
+        <v>118</v>
+      </c>
+      <c r="J39" t="s">
+        <v>171</v>
+      </c>
+      <c r="K39" t="s">
+        <v>192</v>
+      </c>
+      <c r="L39">
+        <v>914782</v>
+      </c>
+      <c r="M39" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13">
+      <c r="A40" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40">
+        <v>2026</v>
+      </c>
+      <c r="D40" t="s">
+        <v>15</v>
+      </c>
+      <c r="E40" t="s">
+        <v>16</v>
+      </c>
+      <c r="F40" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" t="s">
+        <v>18</v>
+      </c>
+      <c r="H40" t="s">
+        <v>57</v>
+      </c>
+      <c r="I40" t="s">
+        <v>119</v>
+      </c>
+      <c r="J40" t="s">
+        <v>171</v>
+      </c>
+      <c r="K40" t="s">
+        <v>198</v>
+      </c>
+      <c r="L40">
+        <v>1015962</v>
+      </c>
+      <c r="M40" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13">
+      <c r="A41" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41">
+        <v>2026</v>
+      </c>
+      <c r="D41" t="s">
+        <v>15</v>
+      </c>
+      <c r="E41" t="s">
+        <v>16</v>
+      </c>
+      <c r="F41" t="s">
+        <v>17</v>
+      </c>
+      <c r="G41" t="s">
+        <v>18</v>
+      </c>
+      <c r="H41" t="s">
+        <v>58</v>
+      </c>
+      <c r="I41" t="s">
+        <v>120</v>
+      </c>
+      <c r="J41" t="s">
+        <v>172</v>
+      </c>
+      <c r="K41" t="s">
+        <v>200</v>
+      </c>
+      <c r="L41">
+        <v>1241196</v>
+      </c>
+      <c r="M41" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13">
+      <c r="A42" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42" t="s">
+        <v>14</v>
+      </c>
+      <c r="C42">
+        <v>2026</v>
+      </c>
+      <c r="D42" t="s">
+        <v>15</v>
+      </c>
+      <c r="E42" t="s">
+        <v>16</v>
+      </c>
+      <c r="F42" t="s">
+        <v>17</v>
+      </c>
+      <c r="G42" t="s">
+        <v>18</v>
+      </c>
+      <c r="H42" t="s">
+        <v>59</v>
+      </c>
+      <c r="I42" t="s">
+        <v>121</v>
+      </c>
+      <c r="J42" t="s">
+        <v>172</v>
+      </c>
+      <c r="K42" t="s">
+        <v>194</v>
+      </c>
+      <c r="L42">
+        <v>1513600</v>
+      </c>
+      <c r="M42" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43">
+        <v>2026</v>
+      </c>
+      <c r="D43" t="s">
+        <v>15</v>
+      </c>
+      <c r="E43" t="s">
+        <v>16</v>
+      </c>
+      <c r="F43" t="s">
+        <v>17</v>
+      </c>
+      <c r="G43" t="s">
+        <v>18</v>
+      </c>
+      <c r="H43" t="s">
+        <v>60</v>
+      </c>
+      <c r="I43" t="s">
+        <v>122</v>
+      </c>
+      <c r="J43" t="s">
+        <v>173</v>
+      </c>
+      <c r="K43" t="s">
+        <v>196</v>
+      </c>
+      <c r="L43">
+        <v>1258720</v>
+      </c>
+      <c r="M43" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13">
+      <c r="A44" t="s">
+        <v>13</v>
+      </c>
+      <c r="B44" t="s">
+        <v>14</v>
+      </c>
+      <c r="C44">
+        <v>2026</v>
+      </c>
+      <c r="D44" t="s">
+        <v>15</v>
+      </c>
+      <c r="E44" t="s">
+        <v>16</v>
+      </c>
+      <c r="F44" t="s">
+        <v>17</v>
+      </c>
+      <c r="G44" t="s">
+        <v>18</v>
+      </c>
+      <c r="H44" t="s">
+        <v>61</v>
+      </c>
+      <c r="I44" t="s">
+        <v>123</v>
+      </c>
+      <c r="J44" t="s">
+        <v>173</v>
+      </c>
+      <c r="K44" t="s">
+        <v>202</v>
+      </c>
+      <c r="L44">
+        <v>1176410</v>
+      </c>
+      <c r="M44" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13">
+      <c r="A45" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" t="s">
+        <v>14</v>
+      </c>
+      <c r="C45">
+        <v>2026</v>
+      </c>
+      <c r="D45" t="s">
+        <v>15</v>
+      </c>
+      <c r="E45" t="s">
+        <v>16</v>
+      </c>
+      <c r="F45" t="s">
+        <v>17</v>
+      </c>
+      <c r="G45" t="s">
+        <v>18</v>
+      </c>
+      <c r="H45" t="s">
+        <v>62</v>
+      </c>
+      <c r="I45" t="s">
+        <v>124</v>
+      </c>
+      <c r="J45" t="s">
+        <v>174</v>
+      </c>
+      <c r="K45" t="s">
+        <v>192</v>
+      </c>
+      <c r="L45">
+        <v>955506</v>
+      </c>
+      <c r="M45" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13">
+      <c r="A46" t="s">
+        <v>13</v>
+      </c>
+      <c r="B46" t="s">
+        <v>14</v>
+      </c>
+      <c r="C46">
+        <v>2026</v>
+      </c>
+      <c r="D46" t="s">
+        <v>15</v>
+      </c>
+      <c r="E46" t="s">
+        <v>16</v>
+      </c>
+      <c r="F46" t="s">
+        <v>17</v>
+      </c>
+      <c r="G46" t="s">
+        <v>18</v>
+      </c>
+      <c r="H46" t="s">
+        <v>63</v>
+      </c>
+      <c r="I46" t="s">
+        <v>125</v>
+      </c>
+      <c r="J46" t="s">
+        <v>175</v>
+      </c>
+      <c r="K46" t="s">
+        <v>193</v>
+      </c>
+      <c r="L46">
+        <v>968160</v>
+      </c>
+      <c r="M46" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13">
+      <c r="A47" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47">
+        <v>2026</v>
+      </c>
+      <c r="D47" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47" t="s">
+        <v>16</v>
+      </c>
+      <c r="F47" t="s">
+        <v>17</v>
+      </c>
+      <c r="G47" t="s">
+        <v>18</v>
+      </c>
+      <c r="H47" t="s">
+        <v>64</v>
+      </c>
+      <c r="I47" t="s">
+        <v>126</v>
+      </c>
+      <c r="J47" t="s">
+        <v>176</v>
+      </c>
+      <c r="K47" t="s">
+        <v>193</v>
+      </c>
+      <c r="L47">
+        <v>970660</v>
+      </c>
+      <c r="M47" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13">
+      <c r="A48" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48" t="s">
+        <v>14</v>
+      </c>
+      <c r="C48">
+        <v>2026</v>
+      </c>
+      <c r="D48" t="s">
+        <v>15</v>
+      </c>
+      <c r="E48" t="s">
+        <v>16</v>
+      </c>
+      <c r="F48" t="s">
+        <v>17</v>
+      </c>
+      <c r="G48" t="s">
+        <v>18</v>
+      </c>
+      <c r="H48" t="s">
+        <v>65</v>
+      </c>
+      <c r="I48" t="s">
+        <v>127</v>
+      </c>
+      <c r="J48" t="s">
+        <v>177</v>
+      </c>
+      <c r="K48" t="s">
+        <v>191</v>
+      </c>
+      <c r="L48">
+        <v>1773944</v>
+      </c>
+      <c r="M48" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13">
+      <c r="A49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49">
+        <v>2026</v>
+      </c>
+      <c r="D49" t="s">
+        <v>15</v>
+      </c>
+      <c r="E49" t="s">
+        <v>16</v>
+      </c>
+      <c r="F49" t="s">
+        <v>17</v>
+      </c>
+      <c r="G49" t="s">
+        <v>18</v>
+      </c>
+      <c r="H49" t="s">
+        <v>66</v>
+      </c>
+      <c r="I49" t="s">
+        <v>128</v>
+      </c>
+      <c r="J49" t="s">
+        <v>178</v>
+      </c>
+      <c r="K49" t="s">
+        <v>201</v>
+      </c>
+      <c r="L49">
+        <v>1524369</v>
+      </c>
+      <c r="M49" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13">
+      <c r="A50" t="s">
+        <v>13</v>
+      </c>
+      <c r="B50" t="s">
+        <v>14</v>
+      </c>
+      <c r="C50">
+        <v>2026</v>
+      </c>
+      <c r="D50" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50" t="s">
+        <v>16</v>
+      </c>
+      <c r="F50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G50" t="s">
+        <v>18</v>
+      </c>
+      <c r="H50" t="s">
+        <v>67</v>
+      </c>
+      <c r="I50" t="s">
+        <v>129</v>
+      </c>
+      <c r="J50" t="s">
+        <v>178</v>
+      </c>
+      <c r="K50" t="s">
+        <v>193</v>
+      </c>
+      <c r="L50">
+        <v>913296</v>
+      </c>
+      <c r="M50" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13">
+      <c r="A51" t="s">
+        <v>13</v>
+      </c>
+      <c r="B51" t="s">
+        <v>14</v>
+      </c>
+      <c r="C51">
+        <v>2026</v>
+      </c>
+      <c r="D51" t="s">
+        <v>15</v>
+      </c>
+      <c r="E51" t="s">
+        <v>16</v>
+      </c>
+      <c r="F51" t="s">
+        <v>17</v>
+      </c>
+      <c r="G51" t="s">
+        <v>18</v>
+      </c>
+      <c r="H51" t="s">
+        <v>68</v>
+      </c>
+      <c r="I51" t="s">
+        <v>130</v>
+      </c>
+      <c r="J51" t="s">
+        <v>178</v>
+      </c>
+      <c r="K51" t="s">
+        <v>199</v>
+      </c>
+      <c r="L51">
+        <v>1658262</v>
+      </c>
+      <c r="M51" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13">
+      <c r="A52" t="s">
+        <v>13</v>
+      </c>
+      <c r="B52" t="s">
+        <v>14</v>
+      </c>
+      <c r="C52">
+        <v>2026</v>
+      </c>
+      <c r="D52" t="s">
+        <v>15</v>
+      </c>
+      <c r="E52" t="s">
+        <v>16</v>
+      </c>
+      <c r="F52" t="s">
+        <v>17</v>
+      </c>
+      <c r="G52" t="s">
+        <v>18</v>
+      </c>
+      <c r="H52" t="s">
+        <v>69</v>
+      </c>
+      <c r="I52" t="s">
+        <v>131</v>
+      </c>
+      <c r="J52" t="s">
+        <v>179</v>
+      </c>
+      <c r="K52" t="s">
+        <v>200</v>
+      </c>
+      <c r="L52">
+        <v>2657794</v>
+      </c>
+      <c r="M52" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13">
+      <c r="A53" t="s">
+        <v>13</v>
+      </c>
+      <c r="B53" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53">
+        <v>2026</v>
+      </c>
+      <c r="D53" t="s">
+        <v>15</v>
+      </c>
+      <c r="E53" t="s">
+        <v>16</v>
+      </c>
+      <c r="F53" t="s">
+        <v>17</v>
+      </c>
+      <c r="G53" t="s">
+        <v>18</v>
+      </c>
+      <c r="H53" t="s">
+        <v>70</v>
+      </c>
+      <c r="I53" t="s">
+        <v>132</v>
+      </c>
+      <c r="J53" t="s">
+        <v>180</v>
+      </c>
+      <c r="K53" t="s">
+        <v>195</v>
+      </c>
+      <c r="L53">
+        <v>4295952</v>
+      </c>
+      <c r="M53" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13">
+      <c r="A54" t="s">
+        <v>13</v>
+      </c>
+      <c r="B54" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54">
+        <v>2026</v>
+      </c>
+      <c r="D54" t="s">
+        <v>15</v>
+      </c>
+      <c r="E54" t="s">
+        <v>16</v>
+      </c>
+      <c r="F54" t="s">
+        <v>17</v>
+      </c>
+      <c r="G54" t="s">
+        <v>18</v>
+      </c>
+      <c r="H54" t="s">
+        <v>71</v>
+      </c>
+      <c r="I54" t="s">
+        <v>133</v>
+      </c>
+      <c r="J54" t="s">
+        <v>181</v>
+      </c>
+      <c r="K54" t="s">
+        <v>194</v>
+      </c>
+      <c r="L54">
+        <v>2276408</v>
+      </c>
+      <c r="M54" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13">
+      <c r="A55" t="s">
+        <v>13</v>
+      </c>
+      <c r="B55" t="s">
+        <v>14</v>
+      </c>
+      <c r="C55">
+        <v>2026</v>
+      </c>
+      <c r="D55" t="s">
+        <v>15</v>
+      </c>
+      <c r="E55" t="s">
+        <v>16</v>
+      </c>
+      <c r="F55" t="s">
+        <v>17</v>
+      </c>
+      <c r="G55" t="s">
+        <v>18</v>
+      </c>
+      <c r="H55" t="s">
+        <v>72</v>
+      </c>
+      <c r="I55" t="s">
+        <v>134</v>
+      </c>
+      <c r="J55" t="s">
+        <v>182</v>
+      </c>
+      <c r="K55" t="s">
+        <v>192</v>
+      </c>
+      <c r="L55">
+        <v>1527990</v>
+      </c>
+      <c r="M55" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13">
+      <c r="A56" t="s">
+        <v>13</v>
+      </c>
+      <c r="B56" t="s">
+        <v>14</v>
+      </c>
+      <c r="C56">
+        <v>2026</v>
+      </c>
+      <c r="D56" t="s">
+        <v>15</v>
+      </c>
+      <c r="E56" t="s">
+        <v>16</v>
+      </c>
+      <c r="F56" t="s">
+        <v>17</v>
+      </c>
+      <c r="G56" t="s">
+        <v>18</v>
+      </c>
+      <c r="H56" t="s">
+        <v>73</v>
+      </c>
+      <c r="I56" t="s">
+        <v>135</v>
+      </c>
+      <c r="J56" t="s">
+        <v>183</v>
+      </c>
+      <c r="K56" t="s">
+        <v>192</v>
+      </c>
+      <c r="L56">
+        <v>956502</v>
+      </c>
+      <c r="M56" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13">
+      <c r="A57" t="s">
+        <v>13</v>
+      </c>
+      <c r="B57" t="s">
+        <v>14</v>
+      </c>
+      <c r="C57">
+        <v>2026</v>
+      </c>
+      <c r="D57" t="s">
+        <v>15</v>
+      </c>
+      <c r="E57" t="s">
+        <v>16</v>
+      </c>
+      <c r="F57" t="s">
+        <v>17</v>
+      </c>
+      <c r="G57" t="s">
+        <v>18</v>
+      </c>
+      <c r="H57" t="s">
+        <v>74</v>
+      </c>
+      <c r="I57" t="s">
+        <v>136</v>
+      </c>
+      <c r="J57" t="s">
+        <v>184</v>
+      </c>
+      <c r="K57" t="s">
+        <v>194</v>
+      </c>
+      <c r="L57">
+        <v>1791600</v>
+      </c>
+      <c r="M57" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13">
+      <c r="A58" t="s">
+        <v>13</v>
+      </c>
+      <c r="B58" t="s">
+        <v>14</v>
+      </c>
+      <c r="C58">
+        <v>2026</v>
+      </c>
+      <c r="D58" t="s">
+        <v>15</v>
+      </c>
+      <c r="E58" t="s">
+        <v>16</v>
+      </c>
+      <c r="F58" t="s">
+        <v>17</v>
+      </c>
+      <c r="G58" t="s">
+        <v>18</v>
+      </c>
+      <c r="H58" t="s">
+        <v>75</v>
+      </c>
+      <c r="I58" t="s">
+        <v>137</v>
+      </c>
+      <c r="J58" t="s">
+        <v>185</v>
+      </c>
+      <c r="K58" t="s">
+        <v>196</v>
+      </c>
+      <c r="L58">
+        <v>1182855</v>
+      </c>
+      <c r="M58" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13">
+      <c r="A59" t="s">
+        <v>13</v>
+      </c>
+      <c r="B59" t="s">
+        <v>14</v>
+      </c>
+      <c r="C59">
+        <v>2026</v>
+      </c>
+      <c r="D59" t="s">
+        <v>15</v>
+      </c>
+      <c r="E59" t="s">
+        <v>16</v>
+      </c>
+      <c r="F59" t="s">
+        <v>17</v>
+      </c>
+      <c r="G59" t="s">
+        <v>18</v>
+      </c>
+      <c r="H59" t="s">
+        <v>76</v>
+      </c>
+      <c r="I59" t="s">
+        <v>138</v>
+      </c>
+      <c r="J59" t="s">
+        <v>186</v>
+      </c>
+      <c r="K59" t="s">
+        <v>194</v>
+      </c>
+      <c r="L59">
+        <v>2812103</v>
+      </c>
+      <c r="M59" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13">
+      <c r="A60" t="s">
+        <v>13</v>
+      </c>
+      <c r="B60" t="s">
+        <v>14</v>
+      </c>
+      <c r="C60">
+        <v>2026</v>
+      </c>
+      <c r="D60" t="s">
+        <v>15</v>
+      </c>
+      <c r="E60" t="s">
+        <v>16</v>
+      </c>
+      <c r="F60" t="s">
+        <v>17</v>
+      </c>
+      <c r="G60" t="s">
+        <v>18</v>
+      </c>
+      <c r="H60" t="s">
+        <v>77</v>
+      </c>
+      <c r="I60" t="s">
+        <v>139</v>
+      </c>
+      <c r="J60" t="s">
+        <v>187</v>
+      </c>
+      <c r="K60" t="s">
+        <v>196</v>
+      </c>
+      <c r="L60">
+        <v>1047586</v>
+      </c>
+      <c r="M60" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13">
+      <c r="A61" t="s">
+        <v>13</v>
+      </c>
+      <c r="B61" t="s">
+        <v>14</v>
+      </c>
+      <c r="C61">
+        <v>2026</v>
+      </c>
+      <c r="D61" t="s">
+        <v>15</v>
+      </c>
+      <c r="E61" t="s">
+        <v>16</v>
+      </c>
+      <c r="F61" t="s">
+        <v>17</v>
+      </c>
+      <c r="G61" t="s">
+        <v>18</v>
+      </c>
+      <c r="H61" t="s">
+        <v>78</v>
+      </c>
+      <c r="I61" t="s">
+        <v>140</v>
+      </c>
+      <c r="J61" t="s">
+        <v>188</v>
+      </c>
+      <c r="K61" t="s">
+        <v>199</v>
+      </c>
+      <c r="L61">
+        <v>1762458</v>
+      </c>
+      <c r="M61" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13">
+      <c r="A62" t="s">
+        <v>13</v>
+      </c>
+      <c r="B62" t="s">
+        <v>14</v>
+      </c>
+      <c r="C62">
+        <v>2026</v>
+      </c>
+      <c r="D62" t="s">
+        <v>15</v>
+      </c>
+      <c r="E62" t="s">
+        <v>16</v>
+      </c>
+      <c r="F62" t="s">
+        <v>17</v>
+      </c>
+      <c r="G62" t="s">
+        <v>18</v>
+      </c>
+      <c r="H62" t="s">
+        <v>79</v>
+      </c>
+      <c r="I62" t="s">
+        <v>141</v>
+      </c>
+      <c r="J62" t="s">
+        <v>189</v>
+      </c>
+      <c r="K62" t="s">
+        <v>199</v>
+      </c>
+      <c r="L62">
+        <v>3126138</v>
+      </c>
+      <c r="M62" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13">
+      <c r="A63" t="s">
+        <v>13</v>
+      </c>
+      <c r="B63" t="s">
+        <v>14</v>
+      </c>
+      <c r="C63">
+        <v>2026</v>
+      </c>
+      <c r="D63" t="s">
+        <v>15</v>
+      </c>
+      <c r="E63" t="s">
+        <v>16</v>
+      </c>
+      <c r="F63" t="s">
+        <v>17</v>
+      </c>
+      <c r="G63" t="s">
+        <v>18</v>
+      </c>
+      <c r="H63" t="s">
         <v>80</v>
       </c>
-      <c r="J32" t="s">
-        <v>108</v>
-      </c>
-      <c r="K32" t="s">
-        <v>112</v>
-      </c>
-      <c r="L32">
-        <v>2600115</v>
-      </c>
-      <c r="M32" t="s">
-        <v>122</v>
+      <c r="I63" t="s">
+        <v>142</v>
+      </c>
+      <c r="J63" t="s">
+        <v>190</v>
+      </c>
+      <c r="K63" t="s">
+        <v>195</v>
+      </c>
+      <c r="L63">
+        <v>1343966</v>
+      </c>
+      <c r="M63" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>